<commit_message>
Add New Splash Screen,User Registration Screen,Login Screen
</commit_message>
<xml_diff>
--- a/assets/File/Demo_Question_File.xlsx
+++ b/assets/File/Demo_Question_File.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\parth\Desktop\Quiz Battle\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\parth\StudioProjects\quiz_battle\assets\File\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{449CAAAA-7466-47DC-B9D1-ABCA9E9DAA7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50DB9B40-B265-443D-806D-17DC63818E89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{BC4C66C7-0EC2-4709-8317-40EC7F61A6D6}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
   <si>
     <t>Question</t>
   </si>
@@ -53,104 +53,47 @@
     <t>Option D</t>
   </si>
   <si>
-    <t>Correct_Answer</t>
-  </si>
-  <si>
-    <t>What does Flutter use for programming?</t>
-  </si>
-  <si>
-    <t>Java</t>
-  </si>
-  <si>
-    <t>Kotlin</t>
-  </si>
-  <si>
-    <t>Dart</t>
-  </si>
-  <si>
-    <t>Python</t>
-  </si>
-  <si>
-    <t>Which widget is used to display text in Flutter?</t>
-  </si>
-  <si>
-    <t>Container</t>
-  </si>
-  <si>
-    <t>Text</t>
-  </si>
-  <si>
-    <t>Column</t>
-  </si>
-  <si>
-    <t>Scaffold</t>
-  </si>
-  <si>
-    <t>What is the capital of India?</t>
-  </si>
-  <si>
-    <t>Mumbai</t>
-  </si>
-  <si>
-    <t>Chennai</t>
-  </si>
-  <si>
-    <t>New Delhi</t>
-  </si>
-  <si>
-    <t>Kolkata</t>
-  </si>
-  <si>
-    <t>Which planet is known as the Red Planet?</t>
-  </si>
-  <si>
-    <t>Earth</t>
-  </si>
-  <si>
-    <t>Mars</t>
-  </si>
-  <si>
-    <t>Jupiter</t>
-  </si>
-  <si>
-    <t>Venus</t>
-  </si>
-  <si>
-    <t>Who invented the telephone?</t>
-  </si>
-  <si>
-    <t>Thomas Edison</t>
-  </si>
-  <si>
-    <t>Alexander Graham Bell</t>
-  </si>
-  <si>
-    <t>Nikola Tesla</t>
-  </si>
-  <si>
-    <t>Albert Einstein</t>
-  </si>
-  <si>
-    <t>Which data type is used for true/false values in Dart?</t>
-  </si>
-  <si>
-    <t>int</t>
-  </si>
-  <si>
-    <t>String</t>
-  </si>
-  <si>
-    <t>bool</t>
-  </si>
-  <si>
-    <t>double</t>
+    <t>Correct Answer</t>
+  </si>
+  <si>
+    <t>What is flutter ?</t>
+  </si>
+  <si>
+    <t>Database</t>
+  </si>
+  <si>
+    <t>UI Toolkit</t>
+  </si>
+  <si>
+    <t>OS</t>
+  </si>
+  <si>
+    <t>Language</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>Who developed Flutter?</t>
+  </si>
+  <si>
+    <t>Apple</t>
+  </si>
+  <si>
+    <t>Google</t>
+  </si>
+  <si>
+    <t>Meta</t>
+  </si>
+  <si>
+    <t>Microsoft</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -163,6 +106,14 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -185,9 +136,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -530,144 +482,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" t="s">
         <v>11</v>
-      </c>
-      <c r="B3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F3" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>19</v>
+      <c r="F4" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>23</v>
-      </c>
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>28</v>
-      </c>
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>34</v>
-      </c>
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>